<commit_message>
Remove build-process language from reports and data; set PDF document author
Drops the resume/interview framing and the 'this session' build artefact from
the written deliverables, renames the confidence tier to source_confirmed, and
regenerates every derived output from the corrected sources.
</commit_message>
<xml_diff>
--- a/excel_model/Campaign_ROI_Simulator.xlsx
+++ b/excel_model/Campaign_ROI_Simulator.xlsx
@@ -918,7 +918,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>-- Campaign assumptions (illustrative — replace before any resume claim) --</t>
+          <t>-- Campaign assumptions (illustrative — replace before using for a spend decision) --</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Illustrative creative production + ad-ops fixed fee; replace with a real rate card figure before any resume claim</t>
+          <t>Illustrative creative production + ad-ops fixed fee; replace with a real rate-card figure before using for a spend decision</t>
         </is>
       </c>
     </row>

</xml_diff>